<commit_message>
Agrega recuadro de logo y datos de empresa en todas las plantillas (Excel y Word)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
+++ b/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,11 @@
     <font>
       <i val="1"/>
       <color rgb="00595959"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00A6A6A6"/>
+      <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
@@ -87,13 +92,45 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <top style="dashed">
+        <color rgb="00A6A6A6"/>
+      </top>
+    </border>
+    <border>
+      <right style="dashed">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="dashed">
+        <color rgb="00A6A6A6"/>
+      </top>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <bottom style="dashed">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="dashed">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <bottom style="dashed">
+        <color rgb="00A6A6A6"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -113,34 +150,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,868 +563,883 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>CONTROL DE INGRESOS Y GASTOS</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>INSERTE SU LOGO
+(clic derecho &gt; Insertar imagen)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="n"/>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Registro diario de movimientos con saldo acumulado</t>
         </is>
       </c>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="7" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Periodo</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Saldo inicial</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Método de pago</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Saldo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="9">
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="14">
         <f>IF(AND(F8="",G8=""),"",$B$5+SUM($F$8:F8)-SUM($G$8:G8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="9">
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="14">
         <f>IF(AND(F9="",G9=""),"",$B$5+SUM($F$8:F9)-SUM($G$8:G9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="9">
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="14">
         <f>IF(AND(F10="",G10=""),"",$B$5+SUM($F$8:F10)-SUM($G$8:G10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="9">
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="14">
         <f>IF(AND(F11="",G11=""),"",$B$5+SUM($F$8:F11)-SUM($G$8:G11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="9">
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="14">
         <f>IF(AND(F12="",G12=""),"",$B$5+SUM($F$8:F12)-SUM($G$8:G12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="9">
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="14">
         <f>IF(AND(F13="",G13=""),"",$B$5+SUM($F$8:F13)-SUM($G$8:G13))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="9">
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="14">
         <f>IF(AND(F14="",G14=""),"",$B$5+SUM($F$8:F14)-SUM($G$8:G14))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="9">
+      <c r="B15" s="13" t="n"/>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
+      <c r="H15" s="14">
         <f>IF(AND(F15="",G15=""),"",$B$5+SUM($F$8:F15)-SUM($G$8:G15))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="9">
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="14">
         <f>IF(AND(F16="",G16=""),"",$B$5+SUM($F$8:F16)-SUM($G$8:G16))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="9">
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
+      <c r="H17" s="14">
         <f>IF(AND(F17="",G17=""),"",$B$5+SUM($F$8:F17)-SUM($G$8:G17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="9">
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="14">
         <f>IF(AND(F18="",G18=""),"",$B$5+SUM($F$8:F18)-SUM($G$8:G18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="9">
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="14">
         <f>IF(AND(F19="",G19=""),"",$B$5+SUM($F$8:F19)-SUM($G$8:G19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="9">
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+      <c r="H20" s="14">
         <f>IF(AND(F20="",G20=""),"",$B$5+SUM($F$8:F20)-SUM($G$8:G20))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="9">
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="14">
         <f>IF(AND(F21="",G21=""),"",$B$5+SUM($F$8:F21)-SUM($G$8:G21))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="9">
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="14">
         <f>IF(AND(F22="",G22=""),"",$B$5+SUM($F$8:F22)-SUM($G$8:G22))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="9">
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="14">
         <f>IF(AND(F23="",G23=""),"",$B$5+SUM($F$8:F23)-SUM($G$8:G23))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="9">
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="14">
         <f>IF(AND(F24="",G24=""),"",$B$5+SUM($F$8:F24)-SUM($G$8:G24))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="9">
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="14">
         <f>IF(AND(F25="",G25=""),"",$B$5+SUM($F$8:F25)-SUM($G$8:G25))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="9">
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="14">
         <f>IF(AND(F26="",G26=""),"",$B$5+SUM($F$8:F26)-SUM($G$8:G26))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="9">
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="14">
         <f>IF(AND(F27="",G27=""),"",$B$5+SUM($F$8:F27)-SUM($G$8:G27))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="9">
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="14">
         <f>IF(AND(F28="",G28=""),"",$B$5+SUM($F$8:F28)-SUM($G$8:G28))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="9">
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="14">
         <f>IF(AND(F29="",G29=""),"",$B$5+SUM($F$8:F29)-SUM($G$8:G29))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="9">
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="14">
         <f>IF(AND(F30="",G30=""),"",$B$5+SUM($F$8:F30)-SUM($G$8:G30))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="9">
+      <c r="B31" s="13" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+      <c r="H31" s="14">
         <f>IF(AND(F31="",G31=""),"",$B$5+SUM($F$8:F31)-SUM($G$8:G31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="9">
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="14">
         <f>IF(AND(F32="",G32=""),"",$B$5+SUM($F$8:F32)-SUM($G$8:G32))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="9">
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="10" t="n"/>
+      <c r="H33" s="14">
         <f>IF(AND(F33="",G33=""),"",$B$5+SUM($F$8:F33)-SUM($G$8:G33))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="n">
+      <c r="A34" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B34" s="8" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="9">
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="14">
         <f>IF(AND(F34="",G34=""),"",$B$5+SUM($F$8:F34)-SUM($G$8:G34))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B35" s="8" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="9">
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="14">
         <f>IF(AND(F35="",G35=""),"",$B$5+SUM($F$8:F35)-SUM($G$8:G35))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n">
+      <c r="A36" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B36" s="8" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="9">
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="14">
         <f>IF(AND(F36="",G36=""),"",$B$5+SUM($F$8:F36)-SUM($G$8:G36))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n">
+      <c r="A37" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="9">
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="14">
         <f>IF(AND(F37="",G37=""),"",$B$5+SUM($F$8:F37)-SUM($G$8:G37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n">
+      <c r="A38" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B38" s="8" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="9">
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="14">
         <f>IF(AND(F38="",G38=""),"",$B$5+SUM($F$8:F38)-SUM($G$8:G38))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="B39" s="8" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="9">
+      <c r="B39" s="13" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="10" t="n"/>
+      <c r="H39" s="14">
         <f>IF(AND(F39="",G39=""),"",$B$5+SUM($F$8:F39)-SUM($G$8:G39))</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="n">
+      <c r="A40" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B40" s="8" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="9">
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+      <c r="H40" s="14">
         <f>IF(AND(F40="",G40=""),"",$B$5+SUM($F$8:F40)-SUM($G$8:G40))</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n">
+      <c r="A41" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B41" s="8" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="9">
+      <c r="B41" s="13" t="n"/>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="14">
         <f>IF(AND(F41="",G41=""),"",$B$5+SUM($F$8:F41)-SUM($G$8:G41))</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n">
+      <c r="A42" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="B42" s="8" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="9">
+      <c r="B42" s="13" t="n"/>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="14">
         <f>IF(AND(F42="",G42=""),"",$B$5+SUM($F$8:F42)-SUM($G$8:G42))</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n">
+      <c r="A43" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B43" s="8" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="9">
+      <c r="B43" s="13" t="n"/>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="14">
         <f>IF(AND(F43="",G43=""),"",$B$5+SUM($F$8:F43)-SUM($G$8:G43))</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="B44" s="8" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="9">
+      <c r="B44" s="13" t="n"/>
+      <c r="C44" s="9" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="14">
         <f>IF(AND(F44="",G44=""),"",$B$5+SUM($F$8:F44)-SUM($G$8:G44))</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B45" s="8" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="9">
+      <c r="B45" s="13" t="n"/>
+      <c r="C45" s="9" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="10" t="n"/>
+      <c r="H45" s="14">
         <f>IF(AND(F45="",G45=""),"",$B$5+SUM($F$8:F45)-SUM($G$8:G45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="n">
+      <c r="A46" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B46" s="8" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="5" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="9">
+      <c r="B46" s="13" t="n"/>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+      <c r="H46" s="14">
         <f>IF(AND(F46="",G46=""),"",$B$5+SUM($F$8:F46)-SUM($G$8:G46))</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B47" s="8" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="9">
+      <c r="B47" s="13" t="n"/>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="14">
         <f>IF(AND(F47="",G47=""),"",$B$5+SUM($F$8:F47)-SUM($G$8:G47))</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n">
+      <c r="A48" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="B48" s="8" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="9">
+      <c r="B48" s="13" t="n"/>
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="10" t="n"/>
+      <c r="H48" s="14">
         <f>IF(AND(F48="",G48=""),"",$B$5+SUM($F$8:F48)-SUM($G$8:G48))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B49" s="8" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="9">
+      <c r="B49" s="13" t="n"/>
+      <c r="C49" s="9" t="n"/>
+      <c r="D49" s="9" t="n"/>
+      <c r="E49" s="9" t="n"/>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="14">
         <f>IF(AND(F49="",G49=""),"",$B$5+SUM($F$8:F49)-SUM($G$8:G49))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="12" t="n">
         <v>43</v>
       </c>
-      <c r="B50" s="8" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="9">
+      <c r="B50" s="13" t="n"/>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="14">
         <f>IF(AND(F50="",G50=""),"",$B$5+SUM($F$8:F50)-SUM($G$8:G50))</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="9">
+      <c r="B51" s="13" t="n"/>
+      <c r="C51" s="9" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="14">
         <f>IF(AND(F51="",G51=""),"",$B$5+SUM($F$8:F51)-SUM($G$8:G51))</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="n">
+      <c r="A52" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="B52" s="8" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="5" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="9">
+      <c r="B52" s="13" t="n"/>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="14">
         <f>IF(AND(F52="",G52=""),"",$B$5+SUM($F$8:F52)-SUM($G$8:G52))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="n">
+      <c r="A53" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="B53" s="8" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="9">
+      <c r="B53" s="13" t="n"/>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="10" t="n"/>
+      <c r="H53" s="14">
         <f>IF(AND(F53="",G53=""),"",$B$5+SUM($F$8:F53)-SUM($G$8:G53))</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="n">
+      <c r="A54" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="B54" s="8" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="5" t="n"/>
-      <c r="G54" s="5" t="n"/>
-      <c r="H54" s="9">
+      <c r="B54" s="13" t="n"/>
+      <c r="C54" s="9" t="n"/>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="10" t="n"/>
+      <c r="H54" s="14">
         <f>IF(AND(F54="",G54=""),"",$B$5+SUM($F$8:F54)-SUM($G$8:G54))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n">
+      <c r="A55" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B55" s="8" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="5" t="n"/>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="9">
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="9" t="n"/>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="F55" s="10" t="n"/>
+      <c r="G55" s="10" t="n"/>
+      <c r="H55" s="14">
         <f>IF(AND(F55="",G55=""),"",$B$5+SUM($F$8:F55)-SUM($G$8:G55))</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n">
+      <c r="A56" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B56" s="8" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="5" t="n"/>
-      <c r="H56" s="9">
+      <c r="B56" s="13" t="n"/>
+      <c r="C56" s="9" t="n"/>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="14">
         <f>IF(AND(F56="",G56=""),"",$B$5+SUM($F$8:F56)-SUM($G$8:G56))</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="n">
+      <c r="A57" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B57" s="8" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="5" t="n"/>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="9">
+      <c r="B57" s="13" t="n"/>
+      <c r="C57" s="9" t="n"/>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="14">
         <f>IF(AND(F57="",G57=""),"",$B$5+SUM($F$8:F57)-SUM($G$8:G57))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="E58" s="10" t="inlineStr">
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F58" s="11">
+      <c r="F58" s="16">
         <f>SUM(F8:F57)</f>
         <v/>
       </c>
-      <c r="G58" s="11">
+      <c r="G58" s="16">
         <f>SUM(G8:G57)</f>
         <v/>
       </c>
-      <c r="H58" s="11">
+      <c r="H58" s="16">
         <f>B5+F58-G58</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G1:H2"/>
     <mergeCell ref="F4:H4"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D8:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1402,7 +1461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1410,71 +1469,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Control de ingresos y gastos</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Guía de uso</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Captura el saldo inicial del periodo en la celda amarilla correspondiente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Registra cada movimiento: fecha, concepto, categoría (lista desplegable) y método de pago.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Escribe el monto en la columna Ingreso o Gasto, nunca en ambas.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>El saldo acumulado y los totales se calculan solos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Imprime en horizontal; el formato ya está ajustado a una hoja.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="16" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Personaliza: en el recuadro punteado de la esquina superior derecha inserta tu logo (Insertar &gt; Imágenes) y captura los datos de tu empresa en las celdas amarillas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Celdas amarillas = captura · Celdas grises = cálculo automático (no modificar).</t>
         </is>

</xml_diff>

<commit_message>
Rediseño con estilo ejecutivo Grupo Canville: portada en cada Excel, paleta azul/petróleo/dorado, pie de página, portadas de venta con collage
Corrige evaluación de desempeño que mostraba 'Deficiente' vacía.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
+++ b/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formato" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formato" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,35 +33,82 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="18"/>
+      <sz val="20"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="005B6B78"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00A6A6A6"/>
       <sz val="8"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001B6B73"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="16"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="000B2A4A"/>
     </font>
     <font>
-      <i val="1"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="26"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00C9D3DB"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B6B73"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9A227"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002B2B2B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="005B6B78"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="008A97A3"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -73,31 +120,45 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="000B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00E6ECF1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E5"/>
+        <fgColor rgb="00FFFCF0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00EEF2F5"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00C9A227"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00C9A227"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -134,57 +195,76 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D3DB"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D3DB"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D3DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D3DB"/>
       </bottom>
+    </border>
+    <border>
+      <top style="thick">
+        <color rgb="00C9A227"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00C9A227"/>
+      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -547,6 +627,200 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C9A227"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="88" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>GRUPO CANVILLE</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Control de ingresos y gastos</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Formato administrativo editable · México</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n"/>
+      <c r="D5" s="1" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="6" customHeight="1">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>CÓMO USARLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="B11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Captura el saldo inicial del periodo en la celda amarilla correspondiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="B12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Registra cada movimiento: fecha, concepto, categoría (lista desplegable) y método de pago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="B13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Escribe el monto en la columna Ingreso o Gasto, nunca en ambas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="B14" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>El saldo acumulado y los totales se calculan solos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="B15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Imprime en horizontal; el formato ya está ajustado a una hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="B16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Personaliza: en el recuadro punteado de la esquina superior derecha inserta tu logo (Insertar &gt; Imágenes) y captura los datos de tu empresa en las celdas de captura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>LEYENDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Celda de captura: escribe aquí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Cálculo automático: no la modifiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="12" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Encabezados y títulos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>GRUPO CANVILLE · Formatos administrativos · v1.0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000B2A4A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -563,36 +837,41 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="44" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>CONTROL DE INGRESOS Y GASTOS</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>INSERTE SU LOGO
 (clic derecho &gt; Insertar imagen)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="n"/>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="H1" s="17" t="n"/>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Registro diario de movimientos con saldo acumulado</t>
         </is>
       </c>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="7" t="n"/>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="20" t="n"/>
+      <c r="H2" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
@@ -600,7 +879,7 @@
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="9" t="n"/>
       <c r="D4" s="9" t="n"/>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Periodo</t>
         </is>
@@ -610,824 +889,824 @@
       <c r="H4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Saldo inicial</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="23" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Método de pago</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>Saldo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="13" t="n"/>
+      <c r="B8" s="25" t="n"/>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="9" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="14">
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="26">
         <f>IF(AND(F8="",G8=""),"",$B$5+SUM($F$8:F8)-SUM($G$8:G8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="13" t="n"/>
+      <c r="B9" s="25" t="n"/>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="9" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="14">
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="26">
         <f>IF(AND(F9="",G9=""),"",$B$5+SUM($F$8:F9)-SUM($G$8:G9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="13" t="n"/>
+      <c r="B10" s="25" t="n"/>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="9" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="14">
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="26">
         <f>IF(AND(F10="",G10=""),"",$B$5+SUM($F$8:F10)-SUM($G$8:G10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="13" t="n"/>
+      <c r="B11" s="25" t="n"/>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="14">
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="26">
         <f>IF(AND(F11="",G11=""),"",$B$5+SUM($F$8:F11)-SUM($G$8:G11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="13" t="n"/>
+      <c r="B12" s="25" t="n"/>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="14">
+      <c r="F12" s="23" t="n"/>
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="26">
         <f>IF(AND(F12="",G12=""),"",$B$5+SUM($F$8:F12)-SUM($G$8:G12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="13" t="n"/>
+      <c r="B13" s="25" t="n"/>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="14">
+      <c r="F13" s="23" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="26">
         <f>IF(AND(F13="",G13=""),"",$B$5+SUM($F$8:F13)-SUM($G$8:G13))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="13" t="n"/>
+      <c r="B14" s="25" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="14">
+      <c r="F14" s="23" t="n"/>
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="26">
         <f>IF(AND(F14="",G14=""),"",$B$5+SUM($F$8:F14)-SUM($G$8:G14))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="13" t="n"/>
+      <c r="B15" s="25" t="n"/>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="9" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="14">
+      <c r="F15" s="23" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="26">
         <f>IF(AND(F15="",G15=""),"",$B$5+SUM($F$8:F15)-SUM($G$8:G15))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="13" t="n"/>
+      <c r="B16" s="25" t="n"/>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="14">
+      <c r="F16" s="23" t="n"/>
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="26">
         <f>IF(AND(F16="",G16=""),"",$B$5+SUM($F$8:F16)-SUM($G$8:G16))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="13" t="n"/>
+      <c r="B17" s="25" t="n"/>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="9" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="14">
+      <c r="F17" s="23" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="26">
         <f>IF(AND(F17="",G17=""),"",$B$5+SUM($F$8:F17)-SUM($G$8:G17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="13" t="n"/>
+      <c r="B18" s="25" t="n"/>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="9" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="14">
+      <c r="F18" s="23" t="n"/>
+      <c r="G18" s="23" t="n"/>
+      <c r="H18" s="26">
         <f>IF(AND(F18="",G18=""),"",$B$5+SUM($F$8:F18)-SUM($G$8:G18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n">
+      <c r="A19" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="13" t="n"/>
+      <c r="B19" s="25" t="n"/>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="9" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="14">
+      <c r="F19" s="23" t="n"/>
+      <c r="G19" s="23" t="n"/>
+      <c r="H19" s="26">
         <f>IF(AND(F19="",G19=""),"",$B$5+SUM($F$8:F19)-SUM($G$8:G19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="13" t="n"/>
+      <c r="B20" s="25" t="n"/>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="14">
+      <c r="F20" s="23" t="n"/>
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="26">
         <f>IF(AND(F20="",G20=""),"",$B$5+SUM($F$8:F20)-SUM($G$8:G20))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="13" t="n"/>
+      <c r="B21" s="25" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="9" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="14">
+      <c r="F21" s="23" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="26">
         <f>IF(AND(F21="",G21=""),"",$B$5+SUM($F$8:F21)-SUM($G$8:G21))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="13" t="n"/>
+      <c r="B22" s="25" t="n"/>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="14">
+      <c r="F22" s="23" t="n"/>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="26">
         <f>IF(AND(F22="",G22=""),"",$B$5+SUM($F$8:F22)-SUM($G$8:G22))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="13" t="n"/>
+      <c r="B23" s="25" t="n"/>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="14">
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="26">
         <f>IF(AND(F23="",G23=""),"",$B$5+SUM($F$8:F23)-SUM($G$8:G23))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="13" t="n"/>
+      <c r="B24" s="25" t="n"/>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="14">
+      <c r="F24" s="23" t="n"/>
+      <c r="G24" s="23" t="n"/>
+      <c r="H24" s="26">
         <f>IF(AND(F24="",G24=""),"",$B$5+SUM($F$8:F24)-SUM($G$8:G24))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="13" t="n"/>
+      <c r="B25" s="25" t="n"/>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="14">
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="26">
         <f>IF(AND(F25="",G25=""),"",$B$5+SUM($F$8:F25)-SUM($G$8:G25))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="13" t="n"/>
+      <c r="B26" s="25" t="n"/>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="14">
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="26">
         <f>IF(AND(F26="",G26=""),"",$B$5+SUM($F$8:F26)-SUM($G$8:G26))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n">
+      <c r="A27" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="13" t="n"/>
+      <c r="B27" s="25" t="n"/>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="10" t="n"/>
-      <c r="H27" s="14">
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="26">
         <f>IF(AND(F27="",G27=""),"",$B$5+SUM($F$8:F27)-SUM($G$8:G27))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B28" s="13" t="n"/>
+      <c r="B28" s="25" t="n"/>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
-      <c r="H28" s="14">
+      <c r="F28" s="23" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="26">
         <f>IF(AND(F28="",G28=""),"",$B$5+SUM($F$8:F28)-SUM($G$8:G28))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n">
+      <c r="A29" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B29" s="13" t="n"/>
+      <c r="B29" s="25" t="n"/>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="14">
+      <c r="F29" s="23" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="26">
         <f>IF(AND(F29="",G29=""),"",$B$5+SUM($F$8:F29)-SUM($G$8:G29))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n">
+      <c r="A30" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="13" t="n"/>
+      <c r="B30" s="25" t="n"/>
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="9" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="14">
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="26">
         <f>IF(AND(F30="",G30=""),"",$B$5+SUM($F$8:F30)-SUM($G$8:G30))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n">
+      <c r="A31" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="13" t="n"/>
+      <c r="B31" s="25" t="n"/>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="9" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="10" t="n"/>
-      <c r="H31" s="14">
+      <c r="F31" s="23" t="n"/>
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="26">
         <f>IF(AND(F31="",G31=""),"",$B$5+SUM($F$8:F31)-SUM($G$8:G31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n">
+      <c r="A32" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B32" s="13" t="n"/>
+      <c r="B32" s="25" t="n"/>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
-      <c r="H32" s="14">
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="26">
         <f>IF(AND(F32="",G32=""),"",$B$5+SUM($F$8:F32)-SUM($G$8:G32))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n">
+      <c r="A33" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B33" s="13" t="n"/>
+      <c r="B33" s="25" t="n"/>
       <c r="C33" s="9" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
-      <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
-      <c r="H33" s="14">
+      <c r="F33" s="23" t="n"/>
+      <c r="G33" s="23" t="n"/>
+      <c r="H33" s="26">
         <f>IF(AND(F33="",G33=""),"",$B$5+SUM($F$8:F33)-SUM($G$8:G33))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n">
+      <c r="A34" s="11" t="n">
         <v>27</v>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="25" t="n"/>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
-      <c r="H34" s="14">
+      <c r="F34" s="23" t="n"/>
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="26">
         <f>IF(AND(F34="",G34=""),"",$B$5+SUM($F$8:F34)-SUM($G$8:G34))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="n">
+      <c r="A35" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B35" s="13" t="n"/>
+      <c r="B35" s="25" t="n"/>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="9" t="n"/>
-      <c r="F35" s="10" t="n"/>
-      <c r="G35" s="10" t="n"/>
-      <c r="H35" s="14">
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="26">
         <f>IF(AND(F35="",G35=""),"",$B$5+SUM($F$8:F35)-SUM($G$8:G35))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n">
+      <c r="A36" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="B36" s="13" t="n"/>
+      <c r="B36" s="25" t="n"/>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9" t="n"/>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
-      <c r="H36" s="14">
+      <c r="F36" s="23" t="n"/>
+      <c r="G36" s="23" t="n"/>
+      <c r="H36" s="26">
         <f>IF(AND(F36="",G36=""),"",$B$5+SUM($F$8:F36)-SUM($G$8:G36))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="n">
+      <c r="A37" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B37" s="13" t="n"/>
+      <c r="B37" s="25" t="n"/>
       <c r="C37" s="9" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
-      <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
-      <c r="H37" s="14">
+      <c r="F37" s="23" t="n"/>
+      <c r="G37" s="23" t="n"/>
+      <c r="H37" s="26">
         <f>IF(AND(F37="",G37=""),"",$B$5+SUM($F$8:F37)-SUM($G$8:G37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="B38" s="13" t="n"/>
+      <c r="B38" s="25" t="n"/>
       <c r="C38" s="9" t="n"/>
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="9" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="14">
+      <c r="F38" s="23" t="n"/>
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="26">
         <f>IF(AND(F38="",G38=""),"",$B$5+SUM($F$8:F38)-SUM($G$8:G38))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="n">
+      <c r="A39" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B39" s="13" t="n"/>
+      <c r="B39" s="25" t="n"/>
       <c r="C39" s="9" t="n"/>
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="9" t="n"/>
-      <c r="F39" s="10" t="n"/>
-      <c r="G39" s="10" t="n"/>
-      <c r="H39" s="14">
+      <c r="F39" s="23" t="n"/>
+      <c r="G39" s="23" t="n"/>
+      <c r="H39" s="26">
         <f>IF(AND(F39="",G39=""),"",$B$5+SUM($F$8:F39)-SUM($G$8:G39))</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n">
+      <c r="A40" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="B40" s="13" t="n"/>
+      <c r="B40" s="25" t="n"/>
       <c r="C40" s="9" t="n"/>
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
-      <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
-      <c r="H40" s="14">
+      <c r="F40" s="23" t="n"/>
+      <c r="G40" s="23" t="n"/>
+      <c r="H40" s="26">
         <f>IF(AND(F40="",G40=""),"",$B$5+SUM($F$8:F40)-SUM($G$8:G40))</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="n">
+      <c r="A41" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B41" s="13" t="n"/>
+      <c r="B41" s="25" t="n"/>
       <c r="C41" s="9" t="n"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="9" t="n"/>
-      <c r="F41" s="10" t="n"/>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="14">
+      <c r="F41" s="23" t="n"/>
+      <c r="G41" s="23" t="n"/>
+      <c r="H41" s="26">
         <f>IF(AND(F41="",G41=""),"",$B$5+SUM($F$8:F41)-SUM($G$8:G41))</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="n">
+      <c r="A42" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B42" s="13" t="n"/>
+      <c r="B42" s="25" t="n"/>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="9" t="n"/>
-      <c r="F42" s="10" t="n"/>
-      <c r="G42" s="10" t="n"/>
-      <c r="H42" s="14">
+      <c r="F42" s="23" t="n"/>
+      <c r="G42" s="23" t="n"/>
+      <c r="H42" s="26">
         <f>IF(AND(F42="",G42=""),"",$B$5+SUM($F$8:F42)-SUM($G$8:G42))</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="n">
+      <c r="A43" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B43" s="13" t="n"/>
+      <c r="B43" s="25" t="n"/>
       <c r="C43" s="9" t="n"/>
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="9" t="n"/>
-      <c r="F43" s="10" t="n"/>
-      <c r="G43" s="10" t="n"/>
-      <c r="H43" s="14">
+      <c r="F43" s="23" t="n"/>
+      <c r="G43" s="23" t="n"/>
+      <c r="H43" s="26">
         <f>IF(AND(F43="",G43=""),"",$B$5+SUM($F$8:F43)-SUM($G$8:G43))</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="B44" s="13" t="n"/>
+      <c r="B44" s="25" t="n"/>
       <c r="C44" s="9" t="n"/>
       <c r="D44" s="9" t="n"/>
       <c r="E44" s="9" t="n"/>
-      <c r="F44" s="10" t="n"/>
-      <c r="G44" s="10" t="n"/>
-      <c r="H44" s="14">
+      <c r="F44" s="23" t="n"/>
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="26">
         <f>IF(AND(F44="",G44=""),"",$B$5+SUM($F$8:F44)-SUM($G$8:G44))</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="n">
+      <c r="A45" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B45" s="13" t="n"/>
+      <c r="B45" s="25" t="n"/>
       <c r="C45" s="9" t="n"/>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="9" t="n"/>
-      <c r="F45" s="10" t="n"/>
-      <c r="G45" s="10" t="n"/>
-      <c r="H45" s="14">
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="26">
         <f>IF(AND(F45="",G45=""),"",$B$5+SUM($F$8:F45)-SUM($G$8:G45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="11" t="n">
         <v>39</v>
       </c>
-      <c r="B46" s="13" t="n"/>
+      <c r="B46" s="25" t="n"/>
       <c r="C46" s="9" t="n"/>
       <c r="D46" s="9" t="n"/>
       <c r="E46" s="9" t="n"/>
-      <c r="F46" s="10" t="n"/>
-      <c r="G46" s="10" t="n"/>
-      <c r="H46" s="14">
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="26">
         <f>IF(AND(F46="",G46=""),"",$B$5+SUM($F$8:F46)-SUM($G$8:G46))</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="n">
+      <c r="A47" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B47" s="13" t="n"/>
+      <c r="B47" s="25" t="n"/>
       <c r="C47" s="9" t="n"/>
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="9" t="n"/>
-      <c r="F47" s="10" t="n"/>
-      <c r="G47" s="10" t="n"/>
-      <c r="H47" s="14">
+      <c r="F47" s="23" t="n"/>
+      <c r="G47" s="23" t="n"/>
+      <c r="H47" s="26">
         <f>IF(AND(F47="",G47=""),"",$B$5+SUM($F$8:F47)-SUM($G$8:G47))</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n">
+      <c r="A48" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="B48" s="13" t="n"/>
+      <c r="B48" s="25" t="n"/>
       <c r="C48" s="9" t="n"/>
       <c r="D48" s="9" t="n"/>
       <c r="E48" s="9" t="n"/>
-      <c r="F48" s="10" t="n"/>
-      <c r="G48" s="10" t="n"/>
-      <c r="H48" s="14">
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="26">
         <f>IF(AND(F48="",G48=""),"",$B$5+SUM($F$8:F48)-SUM($G$8:G48))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="n">
+      <c r="A49" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="B49" s="13" t="n"/>
+      <c r="B49" s="25" t="n"/>
       <c r="C49" s="9" t="n"/>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9" t="n"/>
-      <c r="F49" s="10" t="n"/>
-      <c r="G49" s="10" t="n"/>
-      <c r="H49" s="14">
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="26">
         <f>IF(AND(F49="",G49=""),"",$B$5+SUM($F$8:F49)-SUM($G$8:G49))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="n">
+      <c r="A50" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="B50" s="13" t="n"/>
+      <c r="B50" s="25" t="n"/>
       <c r="C50" s="9" t="n"/>
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="9" t="n"/>
-      <c r="F50" s="10" t="n"/>
-      <c r="G50" s="10" t="n"/>
-      <c r="H50" s="14">
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="23" t="n"/>
+      <c r="H50" s="26">
         <f>IF(AND(F50="",G50=""),"",$B$5+SUM($F$8:F50)-SUM($G$8:G50))</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="n">
+      <c r="A51" s="11" t="n">
         <v>44</v>
       </c>
-      <c r="B51" s="13" t="n"/>
+      <c r="B51" s="25" t="n"/>
       <c r="C51" s="9" t="n"/>
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="9" t="n"/>
-      <c r="F51" s="10" t="n"/>
-      <c r="G51" s="10" t="n"/>
-      <c r="H51" s="14">
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="26">
         <f>IF(AND(F51="",G51=""),"",$B$5+SUM($F$8:F51)-SUM($G$8:G51))</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="n">
+      <c r="A52" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="B52" s="13" t="n"/>
+      <c r="B52" s="25" t="n"/>
       <c r="C52" s="9" t="n"/>
       <c r="D52" s="9" t="n"/>
       <c r="E52" s="9" t="n"/>
-      <c r="F52" s="10" t="n"/>
-      <c r="G52" s="10" t="n"/>
-      <c r="H52" s="14">
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="26">
         <f>IF(AND(F52="",G52=""),"",$B$5+SUM($F$8:F52)-SUM($G$8:G52))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="12" t="n">
+      <c r="A53" s="11" t="n">
         <v>46</v>
       </c>
-      <c r="B53" s="13" t="n"/>
+      <c r="B53" s="25" t="n"/>
       <c r="C53" s="9" t="n"/>
       <c r="D53" s="9" t="n"/>
       <c r="E53" s="9" t="n"/>
-      <c r="F53" s="10" t="n"/>
-      <c r="G53" s="10" t="n"/>
-      <c r="H53" s="14">
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="26">
         <f>IF(AND(F53="",G53=""),"",$B$5+SUM($F$8:F53)-SUM($G$8:G53))</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n">
+      <c r="A54" s="11" t="n">
         <v>47</v>
       </c>
-      <c r="B54" s="13" t="n"/>
+      <c r="B54" s="25" t="n"/>
       <c r="C54" s="9" t="n"/>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
-      <c r="F54" s="10" t="n"/>
-      <c r="G54" s="10" t="n"/>
-      <c r="H54" s="14">
+      <c r="F54" s="23" t="n"/>
+      <c r="G54" s="23" t="n"/>
+      <c r="H54" s="26">
         <f>IF(AND(F54="",G54=""),"",$B$5+SUM($F$8:F54)-SUM($G$8:G54))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="n">
+      <c r="A55" s="11" t="n">
         <v>48</v>
       </c>
-      <c r="B55" s="13" t="n"/>
+      <c r="B55" s="25" t="n"/>
       <c r="C55" s="9" t="n"/>
       <c r="D55" s="9" t="n"/>
       <c r="E55" s="9" t="n"/>
-      <c r="F55" s="10" t="n"/>
-      <c r="G55" s="10" t="n"/>
-      <c r="H55" s="14">
+      <c r="F55" s="23" t="n"/>
+      <c r="G55" s="23" t="n"/>
+      <c r="H55" s="26">
         <f>IF(AND(F55="",G55=""),"",$B$5+SUM($F$8:F55)-SUM($G$8:G55))</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n">
+      <c r="A56" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="B56" s="13" t="n"/>
+      <c r="B56" s="25" t="n"/>
       <c r="C56" s="9" t="n"/>
       <c r="D56" s="9" t="n"/>
       <c r="E56" s="9" t="n"/>
-      <c r="F56" s="10" t="n"/>
-      <c r="G56" s="10" t="n"/>
-      <c r="H56" s="14">
+      <c r="F56" s="23" t="n"/>
+      <c r="G56" s="23" t="n"/>
+      <c r="H56" s="26">
         <f>IF(AND(F56="",G56=""),"",$B$5+SUM($F$8:F56)-SUM($G$8:G56))</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="B57" s="13" t="n"/>
+      <c r="B57" s="25" t="n"/>
       <c r="C57" s="9" t="n"/>
       <c r="D57" s="9" t="n"/>
       <c r="E57" s="9" t="n"/>
-      <c r="F57" s="10" t="n"/>
-      <c r="G57" s="10" t="n"/>
-      <c r="H57" s="14">
+      <c r="F57" s="23" t="n"/>
+      <c r="G57" s="23" t="n"/>
+      <c r="H57" s="26">
         <f>IF(AND(F57="",G57=""),"",$B$5+SUM($F$8:F57)-SUM($G$8:G57))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="E58" s="15" t="inlineStr">
+      <c r="E58" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F58" s="16">
+      <c r="F58" s="28">
         <f>SUM(F8:F57)</f>
         <v/>
       </c>
-      <c r="G58" s="16">
+      <c r="G58" s="28">
         <f>SUM(G8:G57)</f>
         <v/>
       </c>
-      <c r="H58" s="16">
+      <c r="H58" s="28">
         <f>B5+F58-G58</f>
         <v/>
       </c>
@@ -1451,105 +1730,14 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="B1" s="17" t="inlineStr">
-        <is>
-          <t>Control de ingresos y gastos</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Guía de uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>Captura el saldo inicial del periodo en la celda amarilla correspondiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>Registra cada movimiento: fecha, concepto, categoría (lista desplegable) y método de pago.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>Escribe el monto en la columna Ingreso o Gasto, nunca en ambas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>El saldo acumulado y los totales se calculan solos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>Imprime en horizontal; el formato ya está ajustado a una hoja.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>Personaliza: en el recuadro punteado de la esquina superior derecha inserta tu logo (Insertar &gt; Imágenes) y captura los datos de tu empresa en las celdas amarillas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>Celdas amarillas = captura · Celdas grises = cálculo automático (no modificar).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 Página &amp;P&amp;R&amp;8 Impreso: &amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nivel profesional: hojas protegidas, tablero Resumen con gráficas, versiones con datos de ejemplo y portadas con capturas reales
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbwLCqGiq6yuWgXYoX8NSd
</commit_message>
<xml_diff>
--- a/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
+++ b/plantillas/1_Contabilidad_y_Finanzas/01_Control_de_Ingresos_y_Gastos.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formato" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +70,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001B6B73"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000B2A4A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00C9A227"/>
       <sz val="10"/>
     </font>
@@ -111,7 +124,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -138,8 +151,13 @@
         <fgColor rgb="00EEF2F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -208,6 +226,48 @@
       </bottom>
     </border>
     <border>
+      <top style="dashed">
+        <color rgb="00A6A6A6"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="dashed">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D3DB"/>
+      </left>
+      <top style="medium">
+        <color rgb="00C9A227"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00C9D3DB"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C9A227"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D3DB"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="00C9D3DB"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00C9D3DB"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00C9D3DB"/>
+      </bottom>
+    </border>
+    <border>
       <top style="thick">
         <color rgb="00C9A227"/>
       </top>
@@ -221,26 +281,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -255,16 +317,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="7" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="9" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -339,6 +422,229 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gastos por categoría</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!C25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0B2A4A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="0B2A4A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$B$26:$B$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$C$26:$C$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ingresos por categoría</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumen'!G25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="1B6B73"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="1B6B73"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumen'!$F$26:$F$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumen'!$G$26:$G$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4140000" cy="2592000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4140000" cy="2592000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -700,6 +1006,7 @@
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
@@ -713,7 +1020,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Captura el saldo inicial del periodo en la celda amarilla correspondiente.</t>
+          <t>Captura el saldo inicial del periodo en la celda de captura correspondiente.</t>
         </is>
       </c>
     </row>
@@ -767,6 +1074,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
         <is>
@@ -798,6 +1106,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="13" t="n"/>
       <c r="B23" s="13" t="n"/>
@@ -812,6 +1121,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
@@ -870,6 +1180,7 @@
       <c r="G2" s="20" t="n"/>
       <c r="H2" s="21" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -900,6 +1211,7 @@
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="9" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
@@ -943,775 +1255,776 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="25" t="n"/>
+      <c r="B8" s="26" t="n"/>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="23" t="n"/>
       <c r="G8" s="23" t="n"/>
-      <c r="H8" s="26">
+      <c r="H8" s="27">
         <f>IF(AND(F8="",G8=""),"",$B$5+SUM($F$8:F8)-SUM($G$8:G8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="25" t="n"/>
+      <c r="B9" s="26" t="n"/>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="9" t="n"/>
       <c r="F9" s="23" t="n"/>
       <c r="G9" s="23" t="n"/>
-      <c r="H9" s="26">
+      <c r="H9" s="27">
         <f>IF(AND(F9="",G9=""),"",$B$5+SUM($F$8:F9)-SUM($G$8:G9))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="25" t="n"/>
+      <c r="B10" s="26" t="n"/>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="23" t="n"/>
       <c r="G10" s="23" t="n"/>
-      <c r="H10" s="26">
+      <c r="H10" s="27">
         <f>IF(AND(F10="",G10=""),"",$B$5+SUM($F$8:F10)-SUM($G$8:G10))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="25" t="n"/>
+      <c r="B11" s="26" t="n"/>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="9" t="n"/>
       <c r="F11" s="23" t="n"/>
       <c r="G11" s="23" t="n"/>
-      <c r="H11" s="26">
+      <c r="H11" s="27">
         <f>IF(AND(F11="",G11=""),"",$B$5+SUM($F$8:F11)-SUM($G$8:G11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="25" t="n"/>
+      <c r="B12" s="26" t="n"/>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="23" t="n"/>
       <c r="G12" s="23" t="n"/>
-      <c r="H12" s="26">
+      <c r="H12" s="27">
         <f>IF(AND(F12="",G12=""),"",$B$5+SUM($F$8:F12)-SUM($G$8:G12))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="25" t="n"/>
+      <c r="B13" s="26" t="n"/>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="9" t="n"/>
       <c r="F13" s="23" t="n"/>
       <c r="G13" s="23" t="n"/>
-      <c r="H13" s="26">
+      <c r="H13" s="27">
         <f>IF(AND(F13="",G13=""),"",$B$5+SUM($F$8:F13)-SUM($G$8:G13))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="25" t="n"/>
+      <c r="B14" s="26" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
       <c r="F14" s="23" t="n"/>
       <c r="G14" s="23" t="n"/>
-      <c r="H14" s="26">
+      <c r="H14" s="27">
         <f>IF(AND(F14="",G14=""),"",$B$5+SUM($F$8:F14)-SUM($G$8:G14))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="25" t="n"/>
+      <c r="B15" s="26" t="n"/>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="9" t="n"/>
       <c r="F15" s="23" t="n"/>
       <c r="G15" s="23" t="n"/>
-      <c r="H15" s="26">
+      <c r="H15" s="27">
         <f>IF(AND(F15="",G15=""),"",$B$5+SUM($F$8:F15)-SUM($G$8:G15))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="25" t="n"/>
+      <c r="B16" s="26" t="n"/>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n"/>
       <c r="F16" s="23" t="n"/>
       <c r="G16" s="23" t="n"/>
-      <c r="H16" s="26">
+      <c r="H16" s="27">
         <f>IF(AND(F16="",G16=""),"",$B$5+SUM($F$8:F16)-SUM($G$8:G16))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="25" t="n"/>
+      <c r="B17" s="26" t="n"/>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="9" t="n"/>
       <c r="F17" s="23" t="n"/>
       <c r="G17" s="23" t="n"/>
-      <c r="H17" s="26">
+      <c r="H17" s="27">
         <f>IF(AND(F17="",G17=""),"",$B$5+SUM($F$8:F17)-SUM($G$8:G17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="25" t="n"/>
+      <c r="B18" s="26" t="n"/>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="9" t="n"/>
       <c r="F18" s="23" t="n"/>
       <c r="G18" s="23" t="n"/>
-      <c r="H18" s="26">
+      <c r="H18" s="27">
         <f>IF(AND(F18="",G18=""),"",$B$5+SUM($F$8:F18)-SUM($G$8:G18))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="25" t="n"/>
+      <c r="B19" s="26" t="n"/>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="9" t="n"/>
       <c r="F19" s="23" t="n"/>
       <c r="G19" s="23" t="n"/>
-      <c r="H19" s="26">
+      <c r="H19" s="27">
         <f>IF(AND(F19="",G19=""),"",$B$5+SUM($F$8:F19)-SUM($G$8:G19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="25" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="25" t="n"/>
+      <c r="B20" s="26" t="n"/>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n"/>
       <c r="F20" s="23" t="n"/>
       <c r="G20" s="23" t="n"/>
-      <c r="H20" s="26">
+      <c r="H20" s="27">
         <f>IF(AND(F20="",G20=""),"",$B$5+SUM($F$8:F20)-SUM($G$8:G20))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="25" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="25" t="n"/>
+      <c r="B21" s="26" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="9" t="n"/>
       <c r="F21" s="23" t="n"/>
       <c r="G21" s="23" t="n"/>
-      <c r="H21" s="26">
+      <c r="H21" s="27">
         <f>IF(AND(F21="",G21=""),"",$B$5+SUM($F$8:F21)-SUM($G$8:G21))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="25" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="25" t="n"/>
+      <c r="B22" s="26" t="n"/>
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n"/>
       <c r="F22" s="23" t="n"/>
       <c r="G22" s="23" t="n"/>
-      <c r="H22" s="26">
+      <c r="H22" s="27">
         <f>IF(AND(F22="",G22=""),"",$B$5+SUM($F$8:F22)-SUM($G$8:G22))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="25" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="25" t="n"/>
+      <c r="B23" s="26" t="n"/>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="23" t="n"/>
       <c r="G23" s="23" t="n"/>
-      <c r="H23" s="26">
+      <c r="H23" s="27">
         <f>IF(AND(F23="",G23=""),"",$B$5+SUM($F$8:F23)-SUM($G$8:G23))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="25" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="25" t="n"/>
+      <c r="B24" s="26" t="n"/>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="23" t="n"/>
       <c r="G24" s="23" t="n"/>
-      <c r="H24" s="26">
+      <c r="H24" s="27">
         <f>IF(AND(F24="",G24=""),"",$B$5+SUM($F$8:F24)-SUM($G$8:G24))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="25" t="n"/>
+      <c r="B25" s="26" t="n"/>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
       <c r="F25" s="23" t="n"/>
       <c r="G25" s="23" t="n"/>
-      <c r="H25" s="26">
+      <c r="H25" s="27">
         <f>IF(AND(F25="",G25=""),"",$B$5+SUM($F$8:F25)-SUM($G$8:G25))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="25" t="n">
         <v>19</v>
       </c>
-      <c r="B26" s="25" t="n"/>
+      <c r="B26" s="26" t="n"/>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="23" t="n"/>
       <c r="G26" s="23" t="n"/>
-      <c r="H26" s="26">
+      <c r="H26" s="27">
         <f>IF(AND(F26="",G26=""),"",$B$5+SUM($F$8:F26)-SUM($G$8:G26))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="25" t="n"/>
+      <c r="B27" s="26" t="n"/>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="23" t="n"/>
       <c r="G27" s="23" t="n"/>
-      <c r="H27" s="26">
+      <c r="H27" s="27">
         <f>IF(AND(F27="",G27=""),"",$B$5+SUM($F$8:F27)-SUM($G$8:G27))</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="25" t="n">
         <v>21</v>
       </c>
-      <c r="B28" s="25" t="n"/>
+      <c r="B28" s="26" t="n"/>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="23" t="n"/>
       <c r="G28" s="23" t="n"/>
-      <c r="H28" s="26">
+      <c r="H28" s="27">
         <f>IF(AND(F28="",G28=""),"",$B$5+SUM($F$8:F28)-SUM($G$8:G28))</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n">
+      <c r="A29" s="25" t="n">
         <v>22</v>
       </c>
-      <c r="B29" s="25" t="n"/>
+      <c r="B29" s="26" t="n"/>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
       <c r="F29" s="23" t="n"/>
       <c r="G29" s="23" t="n"/>
-      <c r="H29" s="26">
+      <c r="H29" s="27">
         <f>IF(AND(F29="",G29=""),"",$B$5+SUM($F$8:F29)-SUM($G$8:G29))</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="25" t="n">
         <v>23</v>
       </c>
-      <c r="B30" s="25" t="n"/>
+      <c r="B30" s="26" t="n"/>
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="9" t="n"/>
       <c r="F30" s="23" t="n"/>
       <c r="G30" s="23" t="n"/>
-      <c r="H30" s="26">
+      <c r="H30" s="27">
         <f>IF(AND(F30="",G30=""),"",$B$5+SUM($F$8:F30)-SUM($G$8:G30))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="B31" s="25" t="n"/>
+      <c r="B31" s="26" t="n"/>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="9" t="n"/>
       <c r="F31" s="23" t="n"/>
       <c r="G31" s="23" t="n"/>
-      <c r="H31" s="26">
+      <c r="H31" s="27">
         <f>IF(AND(F31="",G31=""),"",$B$5+SUM($F$8:F31)-SUM($G$8:G31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n">
+      <c r="A32" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="B32" s="25" t="n"/>
+      <c r="B32" s="26" t="n"/>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
       <c r="F32" s="23" t="n"/>
       <c r="G32" s="23" t="n"/>
-      <c r="H32" s="26">
+      <c r="H32" s="27">
         <f>IF(AND(F32="",G32=""),"",$B$5+SUM($F$8:F32)-SUM($G$8:G32))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n">
+      <c r="A33" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="B33" s="25" t="n"/>
+      <c r="B33" s="26" t="n"/>
       <c r="C33" s="9" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
       <c r="F33" s="23" t="n"/>
       <c r="G33" s="23" t="n"/>
-      <c r="H33" s="26">
+      <c r="H33" s="27">
         <f>IF(AND(F33="",G33=""),"",$B$5+SUM($F$8:F33)-SUM($G$8:G33))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n">
+      <c r="A34" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="B34" s="25" t="n"/>
+      <c r="B34" s="26" t="n"/>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
       <c r="F34" s="23" t="n"/>
       <c r="G34" s="23" t="n"/>
-      <c r="H34" s="26">
+      <c r="H34" s="27">
         <f>IF(AND(F34="",G34=""),"",$B$5+SUM($F$8:F34)-SUM($G$8:G34))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
+      <c r="A35" s="25" t="n">
         <v>28</v>
       </c>
-      <c r="B35" s="25" t="n"/>
+      <c r="B35" s="26" t="n"/>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="9" t="n"/>
       <c r="F35" s="23" t="n"/>
       <c r="G35" s="23" t="n"/>
-      <c r="H35" s="26">
+      <c r="H35" s="27">
         <f>IF(AND(F35="",G35=""),"",$B$5+SUM($F$8:F35)-SUM($G$8:G35))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="B36" s="25" t="n"/>
+      <c r="B36" s="26" t="n"/>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9" t="n"/>
       <c r="F36" s="23" t="n"/>
       <c r="G36" s="23" t="n"/>
-      <c r="H36" s="26">
+      <c r="H36" s="27">
         <f>IF(AND(F36="",G36=""),"",$B$5+SUM($F$8:F36)-SUM($G$8:G36))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n">
+      <c r="A37" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="B37" s="25" t="n"/>
+      <c r="B37" s="26" t="n"/>
       <c r="C37" s="9" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
       <c r="F37" s="23" t="n"/>
       <c r="G37" s="23" t="n"/>
-      <c r="H37" s="26">
+      <c r="H37" s="27">
         <f>IF(AND(F37="",G37=""),"",$B$5+SUM($F$8:F37)-SUM($G$8:G37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n">
+      <c r="A38" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="B38" s="25" t="n"/>
+      <c r="B38" s="26" t="n"/>
       <c r="C38" s="9" t="n"/>
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="9" t="n"/>
       <c r="F38" s="23" t="n"/>
       <c r="G38" s="23" t="n"/>
-      <c r="H38" s="26">
+      <c r="H38" s="27">
         <f>IF(AND(F38="",G38=""),"",$B$5+SUM($F$8:F38)-SUM($G$8:G38))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n">
+      <c r="A39" s="25" t="n">
         <v>32</v>
       </c>
-      <c r="B39" s="25" t="n"/>
+      <c r="B39" s="26" t="n"/>
       <c r="C39" s="9" t="n"/>
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="9" t="n"/>
       <c r="F39" s="23" t="n"/>
       <c r="G39" s="23" t="n"/>
-      <c r="H39" s="26">
+      <c r="H39" s="27">
         <f>IF(AND(F39="",G39=""),"",$B$5+SUM($F$8:F39)-SUM($G$8:G39))</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n">
+      <c r="A40" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="B40" s="25" t="n"/>
+      <c r="B40" s="26" t="n"/>
       <c r="C40" s="9" t="n"/>
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="23" t="n"/>
       <c r="G40" s="23" t="n"/>
-      <c r="H40" s="26">
+      <c r="H40" s="27">
         <f>IF(AND(F40="",G40=""),"",$B$5+SUM($F$8:F40)-SUM($G$8:G40))</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n">
+      <c r="A41" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="B41" s="25" t="n"/>
+      <c r="B41" s="26" t="n"/>
       <c r="C41" s="9" t="n"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="9" t="n"/>
       <c r="F41" s="23" t="n"/>
       <c r="G41" s="23" t="n"/>
-      <c r="H41" s="26">
+      <c r="H41" s="27">
         <f>IF(AND(F41="",G41=""),"",$B$5+SUM($F$8:F41)-SUM($G$8:G41))</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n">
+      <c r="A42" s="25" t="n">
         <v>35</v>
       </c>
-      <c r="B42" s="25" t="n"/>
+      <c r="B42" s="26" t="n"/>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="9" t="n"/>
       <c r="F42" s="23" t="n"/>
       <c r="G42" s="23" t="n"/>
-      <c r="H42" s="26">
+      <c r="H42" s="27">
         <f>IF(AND(F42="",G42=""),"",$B$5+SUM($F$8:F42)-SUM($G$8:G42))</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
+      <c r="A43" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="B43" s="25" t="n"/>
+      <c r="B43" s="26" t="n"/>
       <c r="C43" s="9" t="n"/>
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="9" t="n"/>
       <c r="F43" s="23" t="n"/>
       <c r="G43" s="23" t="n"/>
-      <c r="H43" s="26">
+      <c r="H43" s="27">
         <f>IF(AND(F43="",G43=""),"",$B$5+SUM($F$8:F43)-SUM($G$8:G43))</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n">
+      <c r="A44" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="B44" s="25" t="n"/>
+      <c r="B44" s="26" t="n"/>
       <c r="C44" s="9" t="n"/>
       <c r="D44" s="9" t="n"/>
       <c r="E44" s="9" t="n"/>
       <c r="F44" s="23" t="n"/>
       <c r="G44" s="23" t="n"/>
-      <c r="H44" s="26">
+      <c r="H44" s="27">
         <f>IF(AND(F44="",G44=""),"",$B$5+SUM($F$8:F44)-SUM($G$8:G44))</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n">
+      <c r="A45" s="25" t="n">
         <v>38</v>
       </c>
-      <c r="B45" s="25" t="n"/>
+      <c r="B45" s="26" t="n"/>
       <c r="C45" s="9" t="n"/>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="9" t="n"/>
       <c r="F45" s="23" t="n"/>
       <c r="G45" s="23" t="n"/>
-      <c r="H45" s="26">
+      <c r="H45" s="27">
         <f>IF(AND(F45="",G45=""),"",$B$5+SUM($F$8:F45)-SUM($G$8:G45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n">
+      <c r="A46" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="B46" s="25" t="n"/>
+      <c r="B46" s="26" t="n"/>
       <c r="C46" s="9" t="n"/>
       <c r="D46" s="9" t="n"/>
       <c r="E46" s="9" t="n"/>
       <c r="F46" s="23" t="n"/>
       <c r="G46" s="23" t="n"/>
-      <c r="H46" s="26">
+      <c r="H46" s="27">
         <f>IF(AND(F46="",G46=""),"",$B$5+SUM($F$8:F46)-SUM($G$8:G46))</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n">
+      <c r="A47" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="B47" s="25" t="n"/>
+      <c r="B47" s="26" t="n"/>
       <c r="C47" s="9" t="n"/>
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="9" t="n"/>
       <c r="F47" s="23" t="n"/>
       <c r="G47" s="23" t="n"/>
-      <c r="H47" s="26">
+      <c r="H47" s="27">
         <f>IF(AND(F47="",G47=""),"",$B$5+SUM($F$8:F47)-SUM($G$8:G47))</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n">
+      <c r="A48" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="B48" s="25" t="n"/>
+      <c r="B48" s="26" t="n"/>
       <c r="C48" s="9" t="n"/>
       <c r="D48" s="9" t="n"/>
       <c r="E48" s="9" t="n"/>
       <c r="F48" s="23" t="n"/>
       <c r="G48" s="23" t="n"/>
-      <c r="H48" s="26">
+      <c r="H48" s="27">
         <f>IF(AND(F48="",G48=""),"",$B$5+SUM($F$8:F48)-SUM($G$8:G48))</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n">
+      <c r="A49" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="B49" s="25" t="n"/>
+      <c r="B49" s="26" t="n"/>
       <c r="C49" s="9" t="n"/>
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="9" t="n"/>
       <c r="F49" s="23" t="n"/>
       <c r="G49" s="23" t="n"/>
-      <c r="H49" s="26">
+      <c r="H49" s="27">
         <f>IF(AND(F49="",G49=""),"",$B$5+SUM($F$8:F49)-SUM($G$8:G49))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n">
+      <c r="A50" s="25" t="n">
         <v>43</v>
       </c>
-      <c r="B50" s="25" t="n"/>
+      <c r="B50" s="26" t="n"/>
       <c r="C50" s="9" t="n"/>
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="9" t="n"/>
       <c r="F50" s="23" t="n"/>
       <c r="G50" s="23" t="n"/>
-      <c r="H50" s="26">
+      <c r="H50" s="27">
         <f>IF(AND(F50="",G50=""),"",$B$5+SUM($F$8:F50)-SUM($G$8:G50))</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
+      <c r="A51" s="25" t="n">
         <v>44</v>
       </c>
-      <c r="B51" s="25" t="n"/>
+      <c r="B51" s="26" t="n"/>
       <c r="C51" s="9" t="n"/>
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="9" t="n"/>
       <c r="F51" s="23" t="n"/>
       <c r="G51" s="23" t="n"/>
-      <c r="H51" s="26">
+      <c r="H51" s="27">
         <f>IF(AND(F51="",G51=""),"",$B$5+SUM($F$8:F51)-SUM($G$8:G51))</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n">
+      <c r="A52" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="B52" s="25" t="n"/>
+      <c r="B52" s="26" t="n"/>
       <c r="C52" s="9" t="n"/>
       <c r="D52" s="9" t="n"/>
       <c r="E52" s="9" t="n"/>
       <c r="F52" s="23" t="n"/>
       <c r="G52" s="23" t="n"/>
-      <c r="H52" s="26">
+      <c r="H52" s="27">
         <f>IF(AND(F52="",G52=""),"",$B$5+SUM($F$8:F52)-SUM($G$8:G52))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n">
+      <c r="A53" s="25" t="n">
         <v>46</v>
       </c>
-      <c r="B53" s="25" t="n"/>
+      <c r="B53" s="26" t="n"/>
       <c r="C53" s="9" t="n"/>
       <c r="D53" s="9" t="n"/>
       <c r="E53" s="9" t="n"/>
       <c r="F53" s="23" t="n"/>
       <c r="G53" s="23" t="n"/>
-      <c r="H53" s="26">
+      <c r="H53" s="27">
         <f>IF(AND(F53="",G53=""),"",$B$5+SUM($F$8:F53)-SUM($G$8:G53))</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n">
+      <c r="A54" s="25" t="n">
         <v>47</v>
       </c>
-      <c r="B54" s="25" t="n"/>
+      <c r="B54" s="26" t="n"/>
       <c r="C54" s="9" t="n"/>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="23" t="n"/>
       <c r="G54" s="23" t="n"/>
-      <c r="H54" s="26">
+      <c r="H54" s="27">
         <f>IF(AND(F54="",G54=""),"",$B$5+SUM($F$8:F54)-SUM($G$8:G54))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="n">
+      <c r="A55" s="25" t="n">
         <v>48</v>
       </c>
-      <c r="B55" s="25" t="n"/>
+      <c r="B55" s="26" t="n"/>
       <c r="C55" s="9" t="n"/>
       <c r="D55" s="9" t="n"/>
       <c r="E55" s="9" t="n"/>
       <c r="F55" s="23" t="n"/>
       <c r="G55" s="23" t="n"/>
-      <c r="H55" s="26">
+      <c r="H55" s="27">
         <f>IF(AND(F55="",G55=""),"",$B$5+SUM($F$8:F55)-SUM($G$8:G55))</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="n">
+      <c r="A56" s="25" t="n">
         <v>49</v>
       </c>
-      <c r="B56" s="25" t="n"/>
+      <c r="B56" s="26" t="n"/>
       <c r="C56" s="9" t="n"/>
       <c r="D56" s="9" t="n"/>
       <c r="E56" s="9" t="n"/>
       <c r="F56" s="23" t="n"/>
       <c r="G56" s="23" t="n"/>
-      <c r="H56" s="26">
+      <c r="H56" s="27">
         <f>IF(AND(F56="",G56=""),"",$B$5+SUM($F$8:F56)-SUM($G$8:G56))</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="n">
+      <c r="A57" s="25" t="n">
         <v>50</v>
       </c>
-      <c r="B57" s="25" t="n"/>
+      <c r="B57" s="26" t="n"/>
       <c r="C57" s="9" t="n"/>
       <c r="D57" s="9" t="n"/>
       <c r="E57" s="9" t="n"/>
       <c r="F57" s="23" t="n"/>
       <c r="G57" s="23" t="n"/>
-      <c r="H57" s="26">
+      <c r="H57" s="27">
         <f>IF(AND(F57="",G57=""),"",$B$5+SUM($F$8:F57)-SUM($G$8:G57))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="E58" s="27" t="inlineStr">
+      <c r="E58" s="28" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F58" s="28">
+      <c r="F58" s="29">
         <f>SUM(F8:F57)</f>
         <v/>
       </c>
-      <c r="G58" s="28">
+      <c r="G58" s="29">
         <f>SUM(G8:G57)</f>
         <v/>
       </c>
-      <c r="H58" s="28">
+      <c r="H58" s="29">
         <f>B5+F58-G58</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B5:D5"/>
@@ -1740,4 +2053,298 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C9A227"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="44" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>RESUMEN DE INGRESOS Y GASTOS</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>INSERTE SU LOGO
+(clic derecho &gt; Insertar imagen)</t>
+        </is>
+      </c>
+      <c r="I1" s="30" t="n"/>
+      <c r="J1" s="17" t="n"/>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Se actualiza solo con lo que captures en la hoja Formato</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="19" t="n"/>
+      <c r="H2" s="20" t="n"/>
+      <c r="I2" s="31" t="n"/>
+      <c r="J2" s="21" t="n"/>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="n"/>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL GASTOS</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="n"/>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>SALDO FINAL</t>
+        </is>
+      </c>
+      <c r="G4" s="33" t="n"/>
+      <c r="H4" s="32" t="inlineStr">
+        <is>
+          <t>MOVIMIENTOS</t>
+        </is>
+      </c>
+      <c r="I4" s="33" t="n"/>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="B5" s="34">
+        <f>Formato!F58</f>
+        <v/>
+      </c>
+      <c r="C5" s="35" t="n"/>
+      <c r="D5" s="34">
+        <f>Formato!G58</f>
+        <v/>
+      </c>
+      <c r="E5" s="35" t="n"/>
+      <c r="F5" s="34">
+        <f>Formato!H58</f>
+        <v/>
+      </c>
+      <c r="G5" s="35" t="n"/>
+      <c r="H5" s="36">
+        <f>SUMPRODUCT(--(((Formato!F8:F57&lt;&gt;"")+(Formato!G8:G57&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="I5" s="35" t="n"/>
+    </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Gasto por categoría</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>Ingreso por categoría</t>
+        </is>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="37" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="C26" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B26,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="G26" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,F26,Formato!$F$8:$F$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="37" t="inlineStr">
+        <is>
+          <t>Renta</t>
+        </is>
+      </c>
+      <c r="C27" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B27,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="G27" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,F27,Formato!$F$8:$F$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="37" t="inlineStr">
+        <is>
+          <t>Servicios (luz/agua/tel)</t>
+        </is>
+      </c>
+      <c r="C28" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B28,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+      <c r="F28" s="37" t="inlineStr">
+        <is>
+          <t>Otros ingresos</t>
+        </is>
+      </c>
+      <c r="G28" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,F28,Formato!$F$8:$F$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>Insumos</t>
+        </is>
+      </c>
+      <c r="C29" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B29,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>Impuestos</t>
+        </is>
+      </c>
+      <c r="C30" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B30,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="37" t="inlineStr">
+        <is>
+          <t>Publicidad</t>
+        </is>
+      </c>
+      <c r="C31" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B31,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="37" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="C32" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B32,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="37" t="inlineStr">
+        <is>
+          <t>Otros gastos</t>
+        </is>
+      </c>
+      <c r="C33" s="27">
+        <f>SUMIF(Formato!$D$8:$D$57,B33,Formato!$G$8:$G$57)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="11">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H1:J2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 Página &amp;P&amp;R&amp;8 Impreso: &amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>